<commit_message>
Add Longstaff-Schwartz LSM, figures, walkthrough notebook, Excel Monte Carlo sheet
- option_pricer/lsm.py: least-squares Monte Carlo for American options, with tests
  against the CRR tree and the Longstaff-Schwartz (2001) benchmark
- docs/greeks.png and docs/monte_carlo.png generated by examples/make_figures.py
- notebooks/walkthrough.ipynb, executed, outputs included
- Excel: new 'Monte Carlo' sheet (values precomputed in Python, native chart)
- README: figures with captions at the top, one section per method with code
  and real outputs, explanation of the 4.4867 vs 4.478 gap

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/option_pricer.xlsx
+++ b/excel/option_pricer.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Pricer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Chart data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Monte Carlo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chart data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="Spot">Pricer!$B$5</definedName>
@@ -26,8 +27,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -101,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -114,6 +116,11 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -348,6 +355,348 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>MC price and 95% interval vs number of paths</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!B4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$B$5:$B$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!C4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="9AA5B1"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$C$5:$C$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="C9CFD6"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$D$5:$D$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="C9CFD6"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$E$5:$E$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!F4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F6FEB"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$F$5:$F$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!G4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="8DB6F5"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$G$5:$G$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Monte Carlo'!H4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="8DB6F5"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Monte Carlo'!$A$5:$A$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Monte Carlo'!$H$5:$H$14</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Number of paths</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="11.5"/>
+          <min val="9.5"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Call price</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -358,6 +707,33 @@
       <rowOff>0</rowOff>
     </from>
     <ext cx="6120000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -964,6 +1340,470 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Monte Carlo convergence, ATM European call (precomputed in Python)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>S=100, K=100, T=1y, r=5%, vol=20%, seed=N (one independent run per row). Static values: re-run python excel/build_workbook.py to refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Paths (N)</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Black-Scholes</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Plain MC</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Plain low 95%</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Plain high 95%</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Antithetic + CV</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Reduced low 95%</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Reduced high 95%</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Std error ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>9.659121000000001</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>8.422088</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>10.896153</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>10.429363</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>10.188309</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>10.670416</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>5.131772</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>9.937773999999999</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>9.058593</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>10.816956</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>10.431302</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>10.254896</v>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>10.607708</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>4.98385</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>10.566744</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>9.903769</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>11.229719</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>10.542943</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>10.426754</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <v>10.659132</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>5.706011</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>10.355161</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>9.952059</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>10.758264</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>10.441539</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>10.365144</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>10.517934</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>5.27654</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>10.362883</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>10.076227</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>10.649538</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>10.40572</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>10.351609</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>10.459831</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>5.297548</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>20000</v>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>10.309091</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>10.106474</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>10.511707</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>10.46782</v>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>10.430487</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>10.505154</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>5.427194</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>10.378517</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>10.25051</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>10.506525</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>10.459275</v>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>10.435707</v>
+      </c>
+      <c r="H11" s="11" t="n">
+        <v>10.482843</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>5.431421</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>10.373513</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>10.282382</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>10.464644</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>10.452088</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>10.43502</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>10.469156</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>5.339385</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>200000</v>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>10.45138</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>10.386896</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>10.515863</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>10.456581</v>
+      </c>
+      <c r="G13" s="11" t="n">
+        <v>10.444478</v>
+      </c>
+      <c r="H13" s="11" t="n">
+        <v>10.468683</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>5.328077</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>10.450584</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>10.450473</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>10.409644</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>10.491302</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>10.454161</v>
+      </c>
+      <c r="G14" s="11" t="n">
+        <v>10.446566</v>
+      </c>
+      <c r="H14" s="11" t="n">
+        <v>10.461756</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>5.375722</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>American put, Longstaff &amp; Schwartz (2001) case: S=36, K=40, r=6%, vol=20%, T=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Std error</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>European put (Black-Scholes)</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>3.844308</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>American put, CRR tree 2,000 steps</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="n">
+        <v>4.486687</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>American put, LSM 100,000 paths, 50 dates</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n">
+        <v>4.475128</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <v>0.00602</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Paper, finite differences (reference grid)</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="n">
+        <v>4.478</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Paper, LSM simulation</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="n">
+        <v>4.472</v>
+      </c>
+      <c r="C43" s="11" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>The tree is stable at 4.4867 from 1,000 to 20,000 steps; the paper's 4.478 comes from a coarser grid. LSM is noisy (s.e. above) and slightly biased low (estimated exercise rule).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -990,575 +1830,575 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12">
+      <c r="A2" s="15">
         <f>Strike*(0.5+0/40)</f>
         <v/>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="15">
         <f>Pricer!$B$16*(A2*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A2/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A2/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="15">
         <f>MAX(Pricer!$B$16*(A2-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12">
+      <c r="A3" s="15">
         <f>Strike*(0.5+1/40)</f>
         <v/>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="15">
         <f>Pricer!$B$16*(A3*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A3/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A3/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="15">
         <f>MAX(Pricer!$B$16*(A3-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12">
+      <c r="A4" s="15">
         <f>Strike*(0.5+2/40)</f>
         <v/>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="15">
         <f>Pricer!$B$16*(A4*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A4/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A4/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="15">
         <f>MAX(Pricer!$B$16*(A4-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12">
+      <c r="A5" s="15">
         <f>Strike*(0.5+3/40)</f>
         <v/>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="15">
         <f>Pricer!$B$16*(A5*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A5/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A5/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="15">
         <f>MAX(Pricer!$B$16*(A5-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12">
+      <c r="A6" s="15">
         <f>Strike*(0.5+4/40)</f>
         <v/>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="15">
         <f>Pricer!$B$16*(A6*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A6/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A6/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="15">
         <f>MAX(Pricer!$B$16*(A6-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12">
+      <c r="A7" s="15">
         <f>Strike*(0.5+5/40)</f>
         <v/>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="15">
         <f>Pricer!$B$16*(A7*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A7/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A7/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="15">
         <f>MAX(Pricer!$B$16*(A7-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12">
+      <c r="A8" s="15">
         <f>Strike*(0.5+6/40)</f>
         <v/>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="15">
         <f>Pricer!$B$16*(A8*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A8/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A8/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="15">
         <f>MAX(Pricer!$B$16*(A8-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12">
+      <c r="A9" s="15">
         <f>Strike*(0.5+7/40)</f>
         <v/>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="15">
         <f>Pricer!$B$16*(A9*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A9/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A9/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="15">
         <f>MAX(Pricer!$B$16*(A9-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12">
+      <c r="A10" s="15">
         <f>Strike*(0.5+8/40)</f>
         <v/>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="15">
         <f>Pricer!$B$16*(A10*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A10/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A10/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="15">
         <f>MAX(Pricer!$B$16*(A10-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12">
+      <c r="A11" s="15">
         <f>Strike*(0.5+9/40)</f>
         <v/>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="15">
         <f>Pricer!$B$16*(A11*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A11/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A11/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="15">
         <f>MAX(Pricer!$B$16*(A11-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12">
+      <c r="A12" s="15">
         <f>Strike*(0.5+10/40)</f>
         <v/>
       </c>
-      <c r="B12" s="12">
+      <c r="B12" s="15">
         <f>Pricer!$B$16*(A12*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A12/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A12/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="15">
         <f>MAX(Pricer!$B$16*(A12-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12">
+      <c r="A13" s="15">
         <f>Strike*(0.5+11/40)</f>
         <v/>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="15">
         <f>Pricer!$B$16*(A13*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A13/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A13/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="15">
         <f>MAX(Pricer!$B$16*(A13-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12">
+      <c r="A14" s="15">
         <f>Strike*(0.5+12/40)</f>
         <v/>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="15">
         <f>Pricer!$B$16*(A14*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A14/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A14/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="15">
         <f>MAX(Pricer!$B$16*(A14-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12">
+      <c r="A15" s="15">
         <f>Strike*(0.5+13/40)</f>
         <v/>
       </c>
-      <c r="B15" s="12">
+      <c r="B15" s="15">
         <f>Pricer!$B$16*(A15*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A15/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A15/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="15">
         <f>MAX(Pricer!$B$16*(A15-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12">
+      <c r="A16" s="15">
         <f>Strike*(0.5+14/40)</f>
         <v/>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="15">
         <f>Pricer!$B$16*(A16*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A16/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A16/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="15">
         <f>MAX(Pricer!$B$16*(A16-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12">
+      <c r="A17" s="15">
         <f>Strike*(0.5+15/40)</f>
         <v/>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="15">
         <f>Pricer!$B$16*(A17*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A17/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A17/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="15">
         <f>MAX(Pricer!$B$16*(A17-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12">
+      <c r="A18" s="15">
         <f>Strike*(0.5+16/40)</f>
         <v/>
       </c>
-      <c r="B18" s="12">
+      <c r="B18" s="15">
         <f>Pricer!$B$16*(A18*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A18/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A18/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="15">
         <f>MAX(Pricer!$B$16*(A18-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12">
+      <c r="A19" s="15">
         <f>Strike*(0.5+17/40)</f>
         <v/>
       </c>
-      <c r="B19" s="12">
+      <c r="B19" s="15">
         <f>Pricer!$B$16*(A19*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A19/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A19/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="15">
         <f>MAX(Pricer!$B$16*(A19-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12">
+      <c r="A20" s="15">
         <f>Strike*(0.5+18/40)</f>
         <v/>
       </c>
-      <c r="B20" s="12">
+      <c r="B20" s="15">
         <f>Pricer!$B$16*(A20*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A20/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A20/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="15">
         <f>MAX(Pricer!$B$16*(A20-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12">
+      <c r="A21" s="15">
         <f>Strike*(0.5+19/40)</f>
         <v/>
       </c>
-      <c r="B21" s="12">
+      <c r="B21" s="15">
         <f>Pricer!$B$16*(A21*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A21/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A21/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="15">
         <f>MAX(Pricer!$B$16*(A21-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12">
+      <c r="A22" s="15">
         <f>Strike*(0.5+20/40)</f>
         <v/>
       </c>
-      <c r="B22" s="12">
+      <c r="B22" s="15">
         <f>Pricer!$B$16*(A22*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A22/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A22/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="15">
         <f>MAX(Pricer!$B$16*(A22-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12">
+      <c r="A23" s="15">
         <f>Strike*(0.5+21/40)</f>
         <v/>
       </c>
-      <c r="B23" s="12">
+      <c r="B23" s="15">
         <f>Pricer!$B$16*(A23*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A23/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A23/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="15">
         <f>MAX(Pricer!$B$16*(A23-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12">
+      <c r="A24" s="15">
         <f>Strike*(0.5+22/40)</f>
         <v/>
       </c>
-      <c r="B24" s="12">
+      <c r="B24" s="15">
         <f>Pricer!$B$16*(A24*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A24/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A24/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="15">
         <f>MAX(Pricer!$B$16*(A24-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12">
+      <c r="A25" s="15">
         <f>Strike*(0.5+23/40)</f>
         <v/>
       </c>
-      <c r="B25" s="12">
+      <c r="B25" s="15">
         <f>Pricer!$B$16*(A25*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A25/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A25/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C25" s="12">
+      <c r="C25" s="15">
         <f>MAX(Pricer!$B$16*(A25-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12">
+      <c r="A26" s="15">
         <f>Strike*(0.5+24/40)</f>
         <v/>
       </c>
-      <c r="B26" s="12">
+      <c r="B26" s="15">
         <f>Pricer!$B$16*(A26*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A26/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A26/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C26" s="12">
+      <c r="C26" s="15">
         <f>MAX(Pricer!$B$16*(A26-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12">
+      <c r="A27" s="15">
         <f>Strike*(0.5+25/40)</f>
         <v/>
       </c>
-      <c r="B27" s="12">
+      <c r="B27" s="15">
         <f>Pricer!$B$16*(A27*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A27/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A27/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="15">
         <f>MAX(Pricer!$B$16*(A27-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12">
+      <c r="A28" s="15">
         <f>Strike*(0.5+26/40)</f>
         <v/>
       </c>
-      <c r="B28" s="12">
+      <c r="B28" s="15">
         <f>Pricer!$B$16*(A28*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A28/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A28/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C28" s="12">
+      <c r="C28" s="15">
         <f>MAX(Pricer!$B$16*(A28-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12">
+      <c r="A29" s="15">
         <f>Strike*(0.5+27/40)</f>
         <v/>
       </c>
-      <c r="B29" s="12">
+      <c r="B29" s="15">
         <f>Pricer!$B$16*(A29*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A29/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A29/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="15">
         <f>MAX(Pricer!$B$16*(A29-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12">
+      <c r="A30" s="15">
         <f>Strike*(0.5+28/40)</f>
         <v/>
       </c>
-      <c r="B30" s="12">
+      <c r="B30" s="15">
         <f>Pricer!$B$16*(A30*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A30/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A30/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C30" s="12">
+      <c r="C30" s="15">
         <f>MAX(Pricer!$B$16*(A30-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12">
+      <c r="A31" s="15">
         <f>Strike*(0.5+29/40)</f>
         <v/>
       </c>
-      <c r="B31" s="12">
+      <c r="B31" s="15">
         <f>Pricer!$B$16*(A31*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A31/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A31/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C31" s="12">
+      <c r="C31" s="15">
         <f>MAX(Pricer!$B$16*(A31-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12">
+      <c r="A32" s="15">
         <f>Strike*(0.5+30/40)</f>
         <v/>
       </c>
-      <c r="B32" s="12">
+      <c r="B32" s="15">
         <f>Pricer!$B$16*(A32*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A32/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A32/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="15">
         <f>MAX(Pricer!$B$16*(A32-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12">
+      <c r="A33" s="15">
         <f>Strike*(0.5+31/40)</f>
         <v/>
       </c>
-      <c r="B33" s="12">
+      <c r="B33" s="15">
         <f>Pricer!$B$16*(A33*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A33/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A33/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="15">
         <f>MAX(Pricer!$B$16*(A33-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12">
+      <c r="A34" s="15">
         <f>Strike*(0.5+32/40)</f>
         <v/>
       </c>
-      <c r="B34" s="12">
+      <c r="B34" s="15">
         <f>Pricer!$B$16*(A34*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A34/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A34/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="15">
         <f>MAX(Pricer!$B$16*(A34-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="12">
+      <c r="A35" s="15">
         <f>Strike*(0.5+33/40)</f>
         <v/>
       </c>
-      <c r="B35" s="12">
+      <c r="B35" s="15">
         <f>Pricer!$B$16*(A35*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A35/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A35/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="15">
         <f>MAX(Pricer!$B$16*(A35-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12">
+      <c r="A36" s="15">
         <f>Strike*(0.5+34/40)</f>
         <v/>
       </c>
-      <c r="B36" s="12">
+      <c r="B36" s="15">
         <f>Pricer!$B$16*(A36*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A36/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A36/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="15">
         <f>MAX(Pricer!$B$16*(A36-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12">
+      <c r="A37" s="15">
         <f>Strike*(0.5+35/40)</f>
         <v/>
       </c>
-      <c r="B37" s="12">
+      <c r="B37" s="15">
         <f>Pricer!$B$16*(A37*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A37/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A37/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="15">
         <f>MAX(Pricer!$B$16*(A37-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12">
+      <c r="A38" s="15">
         <f>Strike*(0.5+36/40)</f>
         <v/>
       </c>
-      <c r="B38" s="12">
+      <c r="B38" s="15">
         <f>Pricer!$B$16*(A38*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A38/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A38/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="15">
         <f>MAX(Pricer!$B$16*(A38-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12">
+      <c r="A39" s="15">
         <f>Strike*(0.5+37/40)</f>
         <v/>
       </c>
-      <c r="B39" s="12">
+      <c r="B39" s="15">
         <f>Pricer!$B$16*(A39*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A39/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A39/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="15">
         <f>MAX(Pricer!$B$16*(A39-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12">
+      <c r="A40" s="15">
         <f>Strike*(0.5+38/40)</f>
         <v/>
       </c>
-      <c r="B40" s="12">
+      <c r="B40" s="15">
         <f>Pricer!$B$16*(A40*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A40/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A40/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="15">
         <f>MAX(Pricer!$B$16*(A40-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="12">
+      <c r="A41" s="15">
         <f>Strike*(0.5+39/40)</f>
         <v/>
       </c>
-      <c r="B41" s="12">
+      <c r="B41" s="15">
         <f>Pricer!$B$16*(A41*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A41/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A41/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="15">
         <f>MAX(Pricer!$B$16*(A41-Strike),0)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12">
+      <c r="A42" s="15">
         <f>Strike*(0.5+40/40)</f>
         <v/>
       </c>
-      <c r="B42" s="12">
+      <c r="B42" s="15">
         <f>Pricer!$B$16*(A42*EXP(-DivYield*Maturity)*NORMSDIST(Pricer!$B$16*((LN(A42/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity))))-Strike*EXP(-Rate*Maturity)*NORMSDIST(Pricer!$B$16*(((LN(A42/Strike)+(Rate-DivYield+Vol^2/2)*Maturity)/(Vol*SQRT(Maturity)))-Vol*SQRT(Maturity))))</f>
         <v/>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="15">
         <f>MAX(Pricer!$B$16*(A42-Strike),0)</f>
         <v/>
       </c>
@@ -1568,48 +2408,55 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Model: Black-Scholes-Merton for European options, continuous dividend yield.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Uses only long-standing functions (NORMSDIST, LN, EXP), so it works in any Excel version and LibreOffice.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Greeks: vega and rho per 1 percentage point, theta per calendar day (annual / 365).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>American options and Monte Carlo are only in the Python package (option_pricer).</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>The 'Monte Carlo' sheet holds values precomputed in Python (python excel/build_workbook.py); they do not follow the yellow input cells.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>American options are priced in Python (CRR tree, Longstaff-Schwartz); results are on the Monte Carlo sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Optional: vba/BlackScholes.bas adds a =BS_PRICE(...) user function (see README).</t>
         </is>

</xml_diff>